<commit_message>
Synchronizing local state to GitHub
</commit_message>
<xml_diff>
--- a/pre-week-2/homework1.xlsx
+++ b/pre-week-2/homework1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FCF9E12-1268-4E80-8974-8385B48C6D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Store_Data" sheetId="1" r:id="rId1"/>
@@ -132,10 +132,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1458,7 +1457,7 @@
       <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1" s="1">
         <f>AVERAGE(Table1[Monthly Sales])</f>
         <v>49.416666666666664</v>
       </c>

</xml_diff>